<commit_message>
updated Complete and overview Pom files
</commit_message>
<xml_diff>
--- a/src/test/resources/SauceDemoCreds.xlsx
+++ b/src/test/resources/SauceDemoCreds.xlsx
@@ -5,16 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\shashank\Capgemini_Training\abcd\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\shashank\Capgemini_Training\Capgemini-Sprint\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180BE1A7-5F35-4808-9C54-9B44A5BE40BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637945BF-24C7-433C-9046-2A7953143BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{C3E99C08-032C-416B-9CFD-7C33402CD155}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{C3E99C08-032C-416B-9CFD-7C33402CD155}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="16">
   <si>
     <t>usename</t>
   </si>
@@ -59,6 +61,21 @@
   </si>
   <si>
     <t>invalid_password</t>
+  </si>
+  <si>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>lastname</t>
+  </si>
+  <si>
+    <t>zipcode</t>
+  </si>
+  <si>
+    <t>shashank</t>
+  </si>
+  <si>
+    <t>manurey</t>
   </si>
 </sst>
 </file>
@@ -554,4 +571,91 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19E6AEF0-2A21-4A13-B2A8-6387A523F454}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2">
+        <v>123456</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4965910-EC31-49DA-ABA9-F5B92ACDD271}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="13.88671875" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2">
+        <v>123456</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>123456</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>